<commit_message>
Updated SLR data extraction sheet
</commit_message>
<xml_diff>
--- a/SLR/SLR Data Extraction Sheet.xlsx
+++ b/SLR/SLR Data Extraction Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javed\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MS Thesis Imp\basic\SLR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02FAE3CB-6F56-4684-8C25-44DCB0EBB5E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABFB3B59-EF23-4B99-B02B-BC37D330B72E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{411C69F0-4063-4D98-AD8A-ABC4C37A7DA5}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="321">
   <si>
     <t>Paper ID</t>
   </si>
@@ -1891,13 +1891,130 @@
   </si>
   <si>
     <t>Top Challenges Identified</t>
+  </si>
+  <si>
+    <t>[31]</t>
+  </si>
+  <si>
+    <t>[32]</t>
+  </si>
+  <si>
+    <t>[33]</t>
+  </si>
+  <si>
+    <t>[34]</t>
+  </si>
+  <si>
+    <t>[35]</t>
+  </si>
+  <si>
+    <t>[36]</t>
+  </si>
+  <si>
+    <t>[37]</t>
+  </si>
+  <si>
+    <t>[38]</t>
+  </si>
+  <si>
+    <t>[39]</t>
+  </si>
+  <si>
+    <t>[40]</t>
+  </si>
+  <si>
+    <t>[41]</t>
+  </si>
+  <si>
+    <t>[42]</t>
+  </si>
+  <si>
+    <t>[43]</t>
+  </si>
+  <si>
+    <t>[44]</t>
+  </si>
+  <si>
+    <t>[45]</t>
+  </si>
+  <si>
+    <t>[46]</t>
+  </si>
+  <si>
+    <t>[47]</t>
+  </si>
+  <si>
+    <t>[48]</t>
+  </si>
+  <si>
+    <t>[49]</t>
+  </si>
+  <si>
+    <t>[50]</t>
+  </si>
+  <si>
+    <t>[51]</t>
+  </si>
+  <si>
+    <t>[52]</t>
+  </si>
+  <si>
+    <t>[53]</t>
+  </si>
+  <si>
+    <t>[54]</t>
+  </si>
+  <si>
+    <t>[55]</t>
+  </si>
+  <si>
+    <t>[20]</t>
+  </si>
+  <si>
+    <t>[28]</t>
+  </si>
+  <si>
+    <t>[6]</t>
+  </si>
+  <si>
+    <t>[8]</t>
+  </si>
+  <si>
+    <t>[29]</t>
+  </si>
+  <si>
+    <t>[24]</t>
+  </si>
+  <si>
+    <t>[10]</t>
+  </si>
+  <si>
+    <t>[30]</t>
+  </si>
+  <si>
+    <t>[25]</t>
+  </si>
+  <si>
+    <t>[26]</t>
+  </si>
+  <si>
+    <t>[27]</t>
+  </si>
+  <si>
+    <t>[9]</t>
+  </si>
+  <si>
+    <t>[21]</t>
+  </si>
+  <si>
+    <t>[22]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1918,6 +2035,12 @@
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1956,24 +2079,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="8">
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1982,6 +2110,18 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2006,10 +2146,10 @@
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
+      <c14:style val="103"/>
     </mc:Choice>
     <mc:Fallback>
-      <c:style val="2"/>
+      <c:style val="3"/>
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
@@ -2038,21 +2178,24 @@
             <a:gradFill rotWithShape="1">
               <a:gsLst>
                 <a:gs pos="0">
-                  <a:schemeClr val="accent2">
+                  <a:schemeClr val="accent1">
+                    <a:shade val="76000"/>
                     <a:satMod val="103000"/>
                     <a:lumMod val="102000"/>
                     <a:tint val="94000"/>
                   </a:schemeClr>
                 </a:gs>
                 <a:gs pos="50000">
-                  <a:schemeClr val="accent2">
+                  <a:schemeClr val="accent1">
+                    <a:shade val="76000"/>
                     <a:satMod val="110000"/>
                     <a:lumMod val="100000"/>
                     <a:shade val="100000"/>
                   </a:schemeClr>
                 </a:gs>
                 <a:gs pos="100000">
-                  <a:schemeClr val="accent2">
+                  <a:schemeClr val="accent1">
+                    <a:shade val="76000"/>
                     <a:lumMod val="99000"/>
                     <a:satMod val="120000"/>
                     <a:shade val="78000"/>
@@ -2191,6 +2334,7 @@
                     <a:gsLst>
                       <a:gs pos="0">
                         <a:schemeClr val="accent1">
+                          <a:tint val="77000"/>
                           <a:satMod val="103000"/>
                           <a:lumMod val="102000"/>
                           <a:tint val="94000"/>
@@ -2198,6 +2342,7 @@
                       </a:gs>
                       <a:gs pos="50000">
                         <a:schemeClr val="accent1">
+                          <a:tint val="77000"/>
                           <a:satMod val="110000"/>
                           <a:lumMod val="100000"/>
                           <a:shade val="100000"/>
@@ -2205,6 +2350,7 @@
                       </a:gs>
                       <a:gs pos="100000">
                         <a:schemeClr val="accent1">
+                          <a:tint val="77000"/>
                           <a:lumMod val="99000"/>
                           <a:satMod val="120000"/>
                           <a:shade val="78000"/>
@@ -2955,67 +3101,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="dk1">
-                    <a:lumMod val="75000"/>
-                    <a:lumOff val="25000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Taxonomy</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-US" baseline="0"/>
-              <a:t> of AI Methods Used</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1">
-                  <a:lumMod val="75000"/>
-                  <a:lumOff val="25000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
+    <c:autoTitleDeleted val="1"/>
     <c:plotArea>
       <c:layout/>
       <c:doughnutChart>
@@ -3052,6 +3138,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-D82D-4B77-B649-12CC14D9C1CD}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -3071,6 +3162,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-D82D-4B77-B649-12CC14D9C1CD}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -3090,6 +3186,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-D82D-4B77-B649-12CC14D9C1CD}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -3109,6 +3210,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-D82D-4B77-B649-12CC14D9C1CD}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="4"/>
@@ -3128,6 +3234,11 @@
                 </a:outerShdw>
               </a:effectLst>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-D82D-4B77-B649-12CC14D9C1CD}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -3320,25 +3431,9 @@
     </c:extLst>
   </c:chart>
   <c:spPr>
-    <a:gradFill flip="none" rotWithShape="1">
-      <a:gsLst>
-        <a:gs pos="0">
-          <a:schemeClr val="lt1"/>
-        </a:gs>
-        <a:gs pos="39000">
-          <a:schemeClr val="lt1"/>
-        </a:gs>
-        <a:gs pos="100000">
-          <a:schemeClr val="lt1">
-            <a:lumMod val="75000"/>
-          </a:schemeClr>
-        </a:gs>
-      </a:gsLst>
-      <a:path path="circle">
-        <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-      </a:path>
-      <a:tileRect/>
-    </a:gradFill>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="dk1">
@@ -3375,10 +3470,10 @@
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="105"/>
+      <c14:style val="103"/>
     </mc:Choice>
     <mc:Fallback>
-      <c:style val="5"/>
+      <c:style val="3"/>
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
@@ -3396,9 +3491,12 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1500" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="all" spc="100" normalizeH="0" baseline="0">
+            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="lt1"/>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
@@ -3431,18 +3529,42 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:pattFill prst="ltUpDiag">
-              <a:fgClr>
-                <a:schemeClr val="accent3"/>
-              </a:fgClr>
-              <a:bgClr>
-                <a:schemeClr val="lt1"/>
-              </a:bgClr>
-            </a:pattFill>
+            <a:gradFill rotWithShape="1">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="103000"/>
+                    <a:lumMod val="102000"/>
+                    <a:tint val="94000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="50000">
+                  <a:schemeClr val="accent1">
+                    <a:satMod val="110000"/>
+                    <a:lumMod val="100000"/>
+                    <a:shade val="100000"/>
+                  </a:schemeClr>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="99000"/>
+                    <a:satMod val="120000"/>
+                    <a:shade val="78000"/>
+                  </a:schemeClr>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="0"/>
+            </a:gradFill>
             <a:ln>
               <a:noFill/>
             </a:ln>
-            <a:effectLst/>
+            <a:effectLst>
+              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+                <a:srgbClr val="000000">
+                  <a:alpha val="63000"/>
+                </a:srgbClr>
+              </a:outerShdw>
+            </a:effectLst>
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:cat>
@@ -3518,7 +3640,7 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:gapWidth val="269"/>
+        <c:gapWidth val="115"/>
         <c:overlap val="-20"/>
         <c:axId val="475947023"/>
         <c:axId val="475945103"/>
@@ -3536,11 +3658,11 @@
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
-          <a:ln w="3175" cap="flat" cmpd="sng" algn="ctr">
+          <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="accent3">
-                <a:lumMod val="60000"/>
-                <a:lumOff val="40000"/>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:round/>
@@ -3552,9 +3674,12 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" spc="150" normalizeH="0" baseline="0">
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="lt1"/>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
@@ -3582,8 +3707,9 @@
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
-                <a:schemeClr val="lt1">
-                  <a:alpha val="25000"/>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:round/>
@@ -3609,7 +3735,10 @@
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="lt1"/>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
@@ -3637,11 +3766,14 @@
   </c:chart>
   <c:spPr>
     <a:solidFill>
-      <a:schemeClr val="accent3"/>
+      <a:schemeClr val="bg1"/>
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
-        <a:schemeClr val="accent3"/>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -3666,42 +3798,8 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinearReversed" id="21">
   <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
 </cs:colorStyle>
 </file>
 
@@ -3786,8 +3884,8 @@
 </file>
 
 <file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinearReversed" id="23">
-  <a:schemeClr val="accent3"/>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinearReversed" id="21">
+  <a:schemeClr val="accent1"/>
 </cs:colorStyle>
 </file>
 
@@ -5397,88 +5495,86 @@
 </file>
 
 <file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="226">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="341">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:defRPr sz="900" b="1" kern="1200"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
   </cs:axisTitle>
   <cs:categoryAxis>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="3175" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="800" kern="1200" cap="all" spc="150" normalizeH="0" baseline="0"/>
+    <cs:defRPr sz="900" kern="1200"/>
   </cs:categoryAxis>
-  <cs:chartArea>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
-        <a:schemeClr val="phClr"/>
+        <a:schemeClr val="bg1"/>
       </a:solidFill>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="phClr"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:defRPr sz="900" kern="1200"/>
   </cs:chartArea>
   <cs:dataLabel>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr">
-          <a:alpha val="70000"/>
-        </a:schemeClr>
-      </a:solidFill>
-    </cs:spPr>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:dataLabel>
   <cs:dataLabelCallout>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <cs:styleClr val="auto"/>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
@@ -5486,7 +5582,10 @@
       </a:solidFill>
       <a:ln>
         <a:solidFill>
-          <a:schemeClr val="phClr"/>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
         </a:solidFill>
       </a:ln>
     </cs:spPr>
@@ -5497,99 +5596,71 @@
   </cs:dataLabelCallout>
   <cs:dataPoint>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:pattFill prst="ltUpDiag">
-        <a:fgClr>
-          <a:schemeClr val="phClr"/>
-        </a:fgClr>
-        <a:bgClr>
-          <a:schemeClr val="lt1"/>
-        </a:bgClr>
-      </a:pattFill>
-    </cs:spPr>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:pattFill prst="ltUpDiag">
-        <a:fgClr>
-          <a:schemeClr val="phClr"/>
-        </a:fgClr>
-        <a:bgClr>
-          <a:schemeClr val="lt1"/>
-        </a:bgClr>
-      </a:pattFill>
-    </cs:spPr>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:effectRef>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="34925" cap="rnd">
         <a:solidFill>
-          <a:schemeClr val="lt1"/>
+          <a:schemeClr val="phClr"/>
         </a:solidFill>
         <a:round/>
       </a:ln>
-      <a:effectLst>
-        <a:outerShdw dist="25400" dir="2700000" algn="tl" rotWithShape="0">
-          <a:schemeClr val="phClr"/>
-        </a:outerShdw>
-      </a:effectLst>
     </cs:spPr>
   </cs:dataPointLine>
   <cs:dataPointMarker>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-      <a:ln w="22225">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="lt1"/>
+          <a:schemeClr val="phClr"/>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointMarkerLayout size="5"/>
   <cs:dataPointWireframe>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="3"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -5601,30 +5672,31 @@
     </cs:spPr>
   </cs:dataPointWireframe>
   <cs:dataTable>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:dataTable>
   <cs:downBar>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
+    <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
@@ -5633,65 +5705,56 @@
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="35000"/>
-          <a:lumOff val="65000"/>
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
         </a:schemeClr>
       </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
     </cs:spPr>
   </cs:downBar>
   <cs:dropLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:prstDash val="dash"/>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:dropLine>
   <cs:errorBar>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
-      <a:effectLst>
-        <a:glow rad="25400">
-          <a:schemeClr val="lt1"/>
-        </a:glow>
-      </a:effectLst>
     </cs:spPr>
   </cs:errorBar>
   <cs:floor>
@@ -5699,23 +5762,22 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:floor>
   <cs:gridlineMajor>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:alpha val="25000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -5723,62 +5785,59 @@
     </cs:spPr>
   </cs:gridlineMajor>
   <cs:gridlineMinor>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:alpha val="10000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:gridlineMinor>
   <cs:hiLoLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:prstDash val="dash"/>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:hiLoLine>
   <cs:leaderLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:leaderLine>
@@ -5787,7 +5846,10 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:legend>
@@ -5796,7 +5858,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:plotArea>
   <cs:plotArea3D>
@@ -5804,24 +5866,25 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:plotArea3D>
   <cs:seriesAxis>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="3175" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -5830,67 +5893,67 @@
     <cs:defRPr sz="900" kern="1200"/>
   </cs:seriesAxis>
   <cs:seriesLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
-            <a:tint val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:defRPr sz="1500" b="1" kern="1200" cap="all" spc="100" normalizeH="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:alpha val="50000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
       </a:ln>
     </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="1" kern="1200" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="lt1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
   </cs:trendline>
   <cs:trendlineLabel>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:trendlineLabel>
   <cs:upBar>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="0"/>
-    </cs:lnRef>
+    <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
@@ -5898,15 +5961,13 @@
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
-        <a:schemeClr val="lt1">
-          <a:lumMod val="95000"/>
-        </a:schemeClr>
+        <a:schemeClr val="lt1"/>
       </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -5917,7 +5978,10 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
@@ -5926,7 +5990,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="lt1"/>
     </cs:fontRef>
   </cs:wall>
 </cs:chartStyle>
@@ -6085,11 +6149,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BAF7BF58-5108-4E9F-BBB8-DC45294BD343}" name="Table1" displayName="Table1" ref="B2:K42" totalsRowShown="0">
   <autoFilter ref="B2:K42" xr:uid="{BAF7BF58-5108-4E9F-BBB8-DC45294BD343}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{F13108BC-856D-4807-A353-343540EB2C2C}" name="Paper ID"/>
-    <tableColumn id="2" xr3:uid="{944FBB7D-42A5-4655-A798-6697959FBEA1}" name="Title" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{68B63363-A6CD-48CA-A383-67B1C2FC62A1}" name="DOI"/>
-    <tableColumn id="4" xr3:uid="{77AD79ED-57F2-44D4-8513-53841FEDA903}" name="Authors"/>
-    <tableColumn id="5" xr3:uid="{398915DC-FA9E-4C6F-A9A6-EA1817DEE472}" name="Year"/>
+    <tableColumn id="1" xr3:uid="{F13108BC-856D-4807-A353-343540EB2C2C}" name="Paper ID" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{944FBB7D-42A5-4655-A798-6697959FBEA1}" name="Title" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{68B63363-A6CD-48CA-A383-67B1C2FC62A1}" name="DOI" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{77AD79ED-57F2-44D4-8513-53841FEDA903}" name="Authors" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{398915DC-FA9E-4C6F-A9A6-EA1817DEE472}" name="Year" dataDxfId="3"/>
     <tableColumn id="7" xr3:uid="{C1FE78AB-51D8-4AEA-91E0-4A0BD7F8A399}" name="Research Contribution Type"/>
     <tableColumn id="8" xr3:uid="{85A5454E-569E-4AD8-90CB-9C6A0DF6C2EB}" name="RQ1: DT Used?" dataDxfId="2"/>
     <tableColumn id="9" xr3:uid="{72798DDB-0A14-4FAA-9524-1090E01DF267}" name="RQ2: AI Used?" dataDxfId="1"/>
@@ -6417,1313 +6481,1315 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F81D26A-F298-454D-8440-DE988CE47416}">
-  <dimension ref="B2:K42"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:K41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="9.6328125" customWidth="1"/>
-    <col min="3" max="3" width="125.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.54296875" customWidth="1"/>
-    <col min="5" max="5" width="179.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25" customWidth="1"/>
-    <col min="8" max="8" width="54.08984375" style="3" customWidth="1"/>
-    <col min="9" max="9" width="46.7265625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="9.6328125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="74.7265625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.54296875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="31.36328125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="8.7265625" style="1"/>
+    <col min="7" max="7" width="14.26953125" customWidth="1"/>
+    <col min="8" max="8" width="54.08984375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="46.7265625" style="2" customWidth="1"/>
     <col min="10" max="10" width="44.453125" customWidth="1"/>
-    <col min="11" max="11" width="46.6328125" style="3" customWidth="1"/>
+    <col min="11" max="11" width="46.6328125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G2" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="J2" t="s">
         <v>6</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="2:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="B3" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="1">
         <v>2024</v>
       </c>
       <c r="G3" t="s">
         <v>127</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="2" t="s">
         <v>130</v>
       </c>
       <c r="J3" t="s">
         <v>131</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="2" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="4" spans="2:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="B4" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="1">
         <v>2025</v>
       </c>
       <c r="G4" t="s">
         <v>127</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="2" t="s">
         <v>133</v>
       </c>
       <c r="J4" t="s">
         <v>131</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="2" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="5" spans="2:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5" s="1" t="s">
+      <c r="B5" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="1">
         <v>2024</v>
       </c>
       <c r="G5" t="s">
         <v>127</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="2" t="s">
         <v>136</v>
       </c>
       <c r="J5" t="s">
         <v>131</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="2" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="6" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B6">
-        <v>4</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="B6" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="1">
         <v>2025</v>
       </c>
       <c r="G6" t="s">
         <v>127</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="K6" s="3" t="s">
+      <c r="K6" s="2" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="7" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B7">
-        <v>5</v>
-      </c>
-      <c r="C7" s="1" t="s">
+      <c r="B7" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="1">
         <v>2025</v>
       </c>
       <c r="G7" t="s">
         <v>127</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="2" t="s">
         <v>143</v>
       </c>
       <c r="J7" t="s">
         <v>131</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="K7" s="2" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="8" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B8">
-        <v>6</v>
-      </c>
-      <c r="C8" s="1" t="s">
+      <c r="B8" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="1">
         <v>2025</v>
       </c>
       <c r="G8" t="s">
         <v>127</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="2" t="s">
         <v>145</v>
       </c>
       <c r="J8" t="s">
         <v>131</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="K8" s="2" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="9" spans="2:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="B9">
-        <v>7</v>
-      </c>
-      <c r="C9" s="1" t="s">
+      <c r="B9" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="1">
         <v>2025</v>
       </c>
       <c r="G9" t="s">
         <v>127</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="I9" s="2" t="s">
         <v>147</v>
       </c>
       <c r="J9" t="s">
         <v>131</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="K9" s="2" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="10" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B10">
-        <v>8</v>
-      </c>
-      <c r="C10" s="1" t="s">
+      <c r="B10" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="1">
         <v>2025</v>
       </c>
       <c r="G10" t="s">
         <v>127</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="I10" s="2" t="s">
         <v>150</v>
       </c>
       <c r="J10" t="s">
         <v>131</v>
       </c>
-      <c r="K10" s="3" t="s">
+      <c r="K10" s="2" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="11" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B11">
-        <v>9</v>
-      </c>
-      <c r="C11" s="1" t="s">
+      <c r="B11" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="1">
         <v>2025</v>
       </c>
       <c r="G11" t="s">
         <v>128</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H11" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="I11" s="2" t="s">
         <v>153</v>
       </c>
       <c r="J11" t="s">
         <v>131</v>
       </c>
-      <c r="K11" s="3" t="s">
+      <c r="K11" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="12" spans="2:11" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B12">
-        <v>10</v>
-      </c>
-      <c r="C12" s="1" t="s">
+    <row r="12" spans="2:11" ht="58" x14ac:dyDescent="0.35">
+      <c r="B12" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="1">
         <v>2025</v>
       </c>
       <c r="G12" t="s">
         <v>127</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="I12" s="2" t="s">
         <v>156</v>
       </c>
       <c r="J12" t="s">
         <v>131</v>
       </c>
-      <c r="K12" s="3" t="s">
+      <c r="K12" s="2" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="13" spans="2:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="B13">
-        <v>11</v>
-      </c>
-      <c r="C13" s="1" t="s">
+      <c r="B13" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="1">
         <v>2025</v>
       </c>
       <c r="G13" t="s">
         <v>128</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="H13" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="I13" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="J13" s="3" t="s">
+      <c r="J13" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="K13" s="3" t="s">
+      <c r="K13" s="2" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="14" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B14">
-        <v>12</v>
-      </c>
-      <c r="C14" s="1" t="s">
+    <row r="14" spans="2:11" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="B14" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="1">
         <v>2025</v>
       </c>
       <c r="G14" t="s">
         <v>127</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="H14" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="2" t="s">
         <v>163</v>
       </c>
       <c r="J14" t="s">
         <v>131</v>
       </c>
-      <c r="K14" s="3" t="s">
+      <c r="K14" s="2" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="15" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B15">
-        <v>13</v>
-      </c>
-      <c r="C15" s="1" t="s">
+      <c r="B15" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="1">
         <v>2025</v>
       </c>
       <c r="G15" t="s">
         <v>127</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="H15" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="I15" s="2" t="s">
         <v>165</v>
       </c>
       <c r="J15" t="s">
         <v>131</v>
       </c>
-      <c r="K15" s="3" t="s">
+      <c r="K15" s="2" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="16" spans="2:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="B16">
-        <v>14</v>
-      </c>
-      <c r="C16" s="1" t="s">
+      <c r="B16" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="1">
         <v>2025</v>
       </c>
       <c r="G16" t="s">
         <v>127</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="H16" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="I16" s="2" t="s">
         <v>168</v>
       </c>
       <c r="J16" t="s">
         <v>131</v>
       </c>
-      <c r="K16" s="3" t="s">
+      <c r="K16" s="2" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="17" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B17">
-        <v>15</v>
-      </c>
-      <c r="C17" s="1" t="s">
+    <row r="17" spans="2:11" ht="87" x14ac:dyDescent="0.35">
+      <c r="B17" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="1">
         <v>2025</v>
       </c>
       <c r="G17" t="s">
         <v>127</v>
       </c>
-      <c r="H17" s="3" t="s">
+      <c r="H17" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="I17" s="3" t="s">
+      <c r="I17" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="J17" s="3" t="s">
+      <c r="J17" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="K17" s="3" t="s">
+      <c r="K17" s="2" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="18" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B18">
-        <v>16</v>
-      </c>
-      <c r="C18" s="1" t="s">
+      <c r="B18" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="1">
         <v>2025</v>
       </c>
       <c r="G18" t="s">
         <v>127</v>
       </c>
-      <c r="H18" s="3" t="s">
+      <c r="H18" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="I18" s="3" t="s">
+      <c r="I18" s="2" t="s">
         <v>174</v>
       </c>
       <c r="J18" t="s">
         <v>131</v>
       </c>
-      <c r="K18" s="3" t="s">
+      <c r="K18" s="2" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="19" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B19">
-        <v>17</v>
-      </c>
-      <c r="C19" s="1" t="s">
+      <c r="B19" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="1">
         <v>2024</v>
       </c>
       <c r="G19" t="s">
         <v>127</v>
       </c>
-      <c r="H19" s="3" t="s">
+      <c r="H19" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="I19" s="3" t="s">
+      <c r="I19" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="J19" s="3" t="s">
+      <c r="J19" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="K19" s="3" t="s">
+      <c r="K19" s="2" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="20" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B20">
-        <v>18</v>
-      </c>
-      <c r="C20" s="1" t="s">
+      <c r="B20" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="1">
         <v>2024</v>
       </c>
       <c r="G20" t="s">
         <v>127</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="H20" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="I20" s="3" t="s">
+      <c r="I20" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="J20" s="3" t="s">
+      <c r="J20" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="K20" s="3" t="s">
+      <c r="K20" s="2" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="21" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B21">
-        <v>19</v>
-      </c>
-      <c r="C21" s="1" t="s">
+      <c r="B21" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="1">
         <v>2024</v>
       </c>
       <c r="G21" t="s">
         <v>127</v>
       </c>
-      <c r="H21" s="3" t="s">
+      <c r="H21" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="I21" s="3" t="s">
+      <c r="I21" s="2" t="s">
         <v>184</v>
       </c>
       <c r="J21" t="s">
         <v>131</v>
       </c>
-      <c r="K21" s="3" t="s">
+      <c r="K21" s="2" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="22" spans="2:11" ht="58" x14ac:dyDescent="0.35">
-      <c r="B22">
-        <v>20</v>
-      </c>
-      <c r="C22" s="1" t="s">
+      <c r="B22" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="1">
         <v>2024</v>
       </c>
       <c r="G22" t="s">
         <v>127</v>
       </c>
-      <c r="H22" s="3" t="s">
+      <c r="H22" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="I22" s="3" t="s">
+      <c r="I22" s="2" t="s">
         <v>187</v>
       </c>
       <c r="J22" t="s">
         <v>131</v>
       </c>
-      <c r="K22" s="3" t="s">
+      <c r="K22" s="2" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="23" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B23">
-        <v>21</v>
-      </c>
-      <c r="C23" s="1" t="s">
+      <c r="B23" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="1">
         <v>2024</v>
       </c>
       <c r="G23" t="s">
         <v>127</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="H23" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="I23" s="3" t="s">
+      <c r="I23" s="2" t="s">
         <v>190</v>
       </c>
       <c r="J23" t="s">
         <v>131</v>
       </c>
-      <c r="K23" s="3" t="s">
+      <c r="K23" s="2" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="24" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B24">
-        <v>22</v>
-      </c>
-      <c r="C24" s="1" t="s">
+      <c r="B24" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="1">
         <v>2024</v>
       </c>
       <c r="G24" t="s">
         <v>128</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="H24" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="I24" s="3" t="s">
+      <c r="I24" s="2" t="s">
         <v>193</v>
       </c>
       <c r="J24" t="s">
         <v>131</v>
       </c>
-      <c r="K24" s="3" t="s">
+      <c r="K24" s="2" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="25" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B25">
-        <v>23</v>
-      </c>
-      <c r="C25" s="1" t="s">
+      <c r="B25" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="1">
         <v>2024</v>
       </c>
       <c r="G25" t="s">
         <v>127</v>
       </c>
-      <c r="H25" s="3" t="s">
+      <c r="H25" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="I25" s="3" t="s">
+      <c r="I25" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="J25" s="3" t="s">
+      <c r="J25" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="K25" s="3" t="s">
+      <c r="K25" s="2" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="26" spans="2:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="B26">
-        <v>24</v>
-      </c>
-      <c r="C26" s="1" t="s">
+      <c r="B26" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="1">
         <v>2023</v>
       </c>
       <c r="G26" t="s">
         <v>127</v>
       </c>
-      <c r="H26" s="3" t="s">
+      <c r="H26" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="I26" s="3" t="s">
+      <c r="I26" s="2" t="s">
         <v>200</v>
       </c>
       <c r="J26" t="s">
         <v>131</v>
       </c>
-      <c r="K26" s="3" t="s">
+      <c r="K26" s="2" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="27" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B27">
-        <v>25</v>
-      </c>
-      <c r="C27" s="1" t="s">
+      <c r="B27" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="1">
         <v>2022</v>
       </c>
       <c r="G27" t="s">
         <v>127</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="H27" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="I27" s="3" t="s">
+      <c r="I27" s="2" t="s">
         <v>203</v>
       </c>
       <c r="J27" t="s">
         <v>131</v>
       </c>
-      <c r="K27" s="3" t="s">
+      <c r="K27" s="2" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="28" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B28">
-        <v>26</v>
-      </c>
-      <c r="C28" s="1" t="s">
+      <c r="B28" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="C28" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="1">
         <v>2022</v>
       </c>
       <c r="G28" t="s">
         <v>127</v>
       </c>
-      <c r="H28" s="3" t="s">
+      <c r="H28" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="I28" s="3" t="s">
+      <c r="I28" s="2" t="s">
         <v>206</v>
       </c>
       <c r="J28" t="s">
         <v>131</v>
       </c>
-      <c r="K28" s="3" t="s">
+      <c r="K28" s="2" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="29" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B29">
-        <v>27</v>
-      </c>
-      <c r="C29" s="1" t="s">
+      <c r="B29" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="1">
         <v>2022</v>
       </c>
       <c r="G29" t="s">
         <v>127</v>
       </c>
-      <c r="H29" s="3" t="s">
+      <c r="H29" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="I29" s="3" t="s">
+      <c r="I29" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="J29" s="3" t="s">
+      <c r="J29" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="K29" s="3" t="s">
+      <c r="K29" s="2" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="30" spans="2:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="B30">
-        <v>28</v>
-      </c>
-      <c r="C30" s="1" t="s">
+      <c r="B30" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="C30" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="1">
         <v>2022</v>
       </c>
       <c r="G30" t="s">
         <v>128</v>
       </c>
-      <c r="H30" s="3" t="s">
+      <c r="H30" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="I30" s="3" t="s">
+      <c r="I30" s="2" t="s">
         <v>213</v>
       </c>
       <c r="J30" t="s">
         <v>131</v>
       </c>
-      <c r="K30" s="3" t="s">
+      <c r="K30" s="2" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="31" spans="2:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="B31">
-        <v>29</v>
-      </c>
-      <c r="C31" s="1" t="s">
+      <c r="B31" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F31">
+      <c r="F31" s="1">
         <v>2022</v>
       </c>
       <c r="G31" t="s">
         <v>127</v>
       </c>
-      <c r="H31" s="3" t="s">
+      <c r="H31" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="I31" s="3" t="s">
+      <c r="I31" s="2" t="s">
         <v>216</v>
       </c>
       <c r="J31" t="s">
         <v>131</v>
       </c>
-      <c r="K31" s="3" t="s">
+      <c r="K31" s="2" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="32" spans="2:11" ht="116" x14ac:dyDescent="0.35">
-      <c r="B32">
-        <v>30</v>
-      </c>
-      <c r="C32" s="1" t="s">
+      <c r="B32" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C32" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="F32">
+      <c r="F32" s="1">
         <v>2021</v>
       </c>
       <c r="G32" t="s">
         <v>127</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="H32" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="I32" s="3" t="s">
+      <c r="I32" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="J32" s="3" t="s">
+      <c r="J32" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="K32" s="3" t="s">
+      <c r="K32" s="2" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="33" spans="2:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="B33">
-        <v>31</v>
-      </c>
-      <c r="C33" s="1" t="s">
+      <c r="B33" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="C33" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="F33">
+      <c r="F33" s="1">
         <v>2021</v>
       </c>
       <c r="G33" t="s">
         <v>127</v>
       </c>
-      <c r="H33" s="3" t="s">
+      <c r="H33" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="I33" s="3" t="s">
+      <c r="I33" s="2" t="s">
         <v>223</v>
       </c>
       <c r="J33" t="s">
         <v>131</v>
       </c>
-      <c r="K33" s="3" t="s">
+      <c r="K33" s="2" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="34" spans="2:11" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="B34">
-        <v>32</v>
-      </c>
-      <c r="C34" s="1" t="s">
+      <c r="B34" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="C34" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="F34">
+      <c r="F34" s="1">
         <v>2021</v>
       </c>
       <c r="G34" t="s">
         <v>127</v>
       </c>
-      <c r="H34" s="3" t="s">
+      <c r="H34" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="I34" s="3" t="s">
+      <c r="I34" s="2" t="s">
         <v>226</v>
       </c>
       <c r="J34" t="s">
         <v>131</v>
       </c>
-      <c r="K34" s="3" t="s">
+      <c r="K34" s="2" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="35" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B35">
-        <v>33</v>
-      </c>
-      <c r="C35" s="1" t="s">
+      <c r="B35" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E35" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="F35">
+      <c r="F35" s="1">
         <v>2021</v>
       </c>
       <c r="G35" t="s">
         <v>127</v>
       </c>
-      <c r="H35" s="3" t="s">
+      <c r="H35" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="I35" s="3" t="s">
+      <c r="I35" s="2" t="s">
         <v>229</v>
       </c>
       <c r="J35" t="s">
         <v>131</v>
       </c>
-      <c r="K35" s="3" t="s">
+      <c r="K35" s="2" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="36" spans="2:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="B36">
-        <v>34</v>
-      </c>
-      <c r="C36" s="1" t="s">
+      <c r="B36" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="C36" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E36" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="F36">
+      <c r="F36" s="1">
         <v>2020</v>
       </c>
       <c r="G36" t="s">
         <v>127</v>
       </c>
-      <c r="H36" s="3" t="s">
+      <c r="H36" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="I36" s="3" t="s">
+      <c r="I36" s="2" t="s">
         <v>232</v>
       </c>
       <c r="J36" t="s">
         <v>131</v>
       </c>
-      <c r="K36" s="3" t="s">
+      <c r="K36" s="2" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="37" spans="2:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="B37">
-        <v>35</v>
-      </c>
-      <c r="C37" s="1" t="s">
+      <c r="B37" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E37" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="1">
         <v>2019</v>
       </c>
       <c r="G37" t="s">
         <v>127</v>
       </c>
-      <c r="H37" s="3" t="s">
+      <c r="H37" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="I37" s="3" t="s">
+      <c r="I37" s="2" t="s">
         <v>235</v>
       </c>
       <c r="J37" t="s">
         <v>131</v>
       </c>
-      <c r="K37" s="3" t="s">
+      <c r="K37" s="2" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="38" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B38">
-        <v>36</v>
-      </c>
-      <c r="C38" s="1" t="s">
+      <c r="B38" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C38" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E38" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="1">
         <v>2018</v>
       </c>
       <c r="G38" t="s">
         <v>128</v>
       </c>
-      <c r="H38" s="3" t="s">
+      <c r="H38" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="I38" s="3" t="s">
+      <c r="I38" s="2" t="s">
         <v>238</v>
       </c>
       <c r="J38" t="s">
         <v>131</v>
       </c>
-      <c r="K38" s="3" t="s">
+      <c r="K38" s="2" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="39" spans="2:11" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B39">
-        <v>37</v>
-      </c>
-      <c r="C39" s="1" t="s">
+      <c r="B39" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E39" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="1">
         <v>2023</v>
       </c>
       <c r="G39" t="s">
         <v>128</v>
       </c>
-      <c r="H39" s="3" t="s">
+      <c r="H39" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="I39" s="3" t="s">
+      <c r="I39" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="J39" s="3" t="s">
+      <c r="J39" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="K39" s="3" t="s">
+      <c r="K39" s="2" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="40" spans="2:11" ht="87" x14ac:dyDescent="0.35">
-      <c r="B40">
-        <v>38</v>
-      </c>
-      <c r="C40" s="1" t="s">
+      <c r="B40" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C40" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E40" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="F40">
+      <c r="F40" s="1">
         <v>2025</v>
       </c>
       <c r="G40" t="s">
         <v>127</v>
       </c>
-      <c r="H40" s="3" t="s">
+      <c r="H40" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="I40" s="3" t="s">
+      <c r="I40" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="J40" s="3" t="s">
+      <c r="J40" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="K40" s="3" t="s">
+      <c r="K40" s="2" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="41" spans="2:11" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="B41">
-        <v>39</v>
-      </c>
-      <c r="C41" s="1" t="s">
+      <c r="B41" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="C41" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="D41" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E41" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="F41">
+      <c r="F41" s="1">
         <v>2026</v>
       </c>
       <c r="G41" t="s">
         <v>127</v>
       </c>
-      <c r="H41" s="3" t="s">
+      <c r="H41" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="I41" s="3" t="s">
+      <c r="I41" s="2" t="s">
         <v>249</v>
       </c>
       <c r="J41" t="s">
         <v>131</v>
       </c>
-      <c r="K41" s="3" t="s">
+      <c r="K41" s="2" t="s">
         <v>250</v>
-      </c>
-    </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B42">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1" xr:uid="{9D3D62E4-E3A7-495F-9AC7-AFADB3865D57}"/>
     <hyperlink ref="D41" r:id="rId2" xr:uid="{B9F84DB3-C4EC-4C0F-9D5E-B0ECAED8C950}"/>
   </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="17" orientation="landscape" r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7932,10 +7998,10 @@
       <c r="B53" t="s">
         <v>268</v>
       </c>
-      <c r="D53" s="4" t="s">
+      <c r="D53" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="E53" s="4" t="s">
+      <c r="E53" s="3" t="s">
         <v>270</v>
       </c>
     </row>
@@ -7943,58 +8009,58 @@
       <c r="B54" t="s">
         <v>281</v>
       </c>
-      <c r="D54" s="4" t="s">
+      <c r="D54" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="E54" s="4">
+      <c r="E54" s="3">
         <v>26</v>
       </c>
     </row>
     <row r="55" spans="2:5" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D55" s="4" t="s">
+      <c r="D55" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="E55" s="4">
+      <c r="E55" s="3">
         <v>17</v>
       </c>
     </row>
     <row r="56" spans="2:5" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D56" s="4" t="s">
+      <c r="D56" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="E56" s="4">
+      <c r="E56" s="3">
         <v>16</v>
       </c>
     </row>
     <row r="57" spans="2:5" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D57" s="4" t="s">
+      <c r="D57" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="E57" s="4">
+      <c r="E57" s="3">
         <v>13</v>
       </c>
     </row>
     <row r="58" spans="2:5" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D58" s="4" t="s">
+      <c r="D58" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="E58" s="4">
+      <c r="E58" s="3">
         <v>12</v>
       </c>
     </row>
     <row r="59" spans="2:5" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D59" s="4" t="s">
+      <c r="D59" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="E59" s="4">
+      <c r="E59" s="3">
         <v>11</v>
       </c>
     </row>
     <row r="60" spans="2:5" ht="70.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D60" s="4" t="s">
+      <c r="D60" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="E60" s="4">
+      <c r="E60" s="3">
         <v>11</v>
       </c>
     </row>

</xml_diff>